<commit_message>
some new features added
</commit_message>
<xml_diff>
--- a/TestData/testData.xlsx
+++ b/TestData/testData.xlsx
@@ -158,7 +158,7 @@
     <t>mrs</t>
   </si>
   <si>
-    <t>test00112233@gmail.com</t>
+    <t>test001122314yoglyo4@gmail.com</t>
   </si>
   <si>
     <t>msedge.exe</t>
@@ -167,7 +167,16 @@
     <t>May</t>
   </si>
   <si>
-    <t>thsirt</t>
+    <t>tshirt</t>
+  </si>
+  <si>
+    <t>test0011443344@gmail.com</t>
+  </si>
+  <si>
+    <t>Sanju</t>
+  </si>
+  <si>
+    <t>dress</t>
   </si>
 </sst>
 </file>
@@ -747,6 +756,50 @@
         <v>39</v>
       </c>
     </row>
+    <row r="4">
+      <c r="K4" t="s">
+        <v>31</v>
+      </c>
+      <c r="L4" t="s">
+        <v>32</v>
+      </c>
+      <c r="M4" t="s">
+        <v>50</v>
+      </c>
+      <c r="N4" t="s">
+        <v>51</v>
+      </c>
+      <c r="O4" t="s">
+        <v>35</v>
+      </c>
+      <c r="P4" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q4">
+        <v>2003</v>
+      </c>
+      <c r="R4" t="s">
+        <v>52</v>
+      </c>
+      <c r="S4">
+        <v>2030</v>
+      </c>
+      <c r="T4">
+        <v>2</v>
+      </c>
+      <c r="U4">
+        <v>123</v>
+      </c>
+      <c r="V4">
+        <v>321654987</v>
+      </c>
+      <c r="W4" t="s">
+        <v>51</v>
+      </c>
+      <c r="X4" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="M2" r:id="rId1"/>

</xml_diff>